<commit_message>
- Pulse DAC logic is now complete.  - The 4-bit adders are verified correct using Excel.    - This revealed 1 tracing error and also 3 XNOR gates that are actually XOR in this case.  - Now including a PDF version of the schematic.
</commit_message>
<xml_diff>
--- a/list of gates updated.xlsx
+++ b/list of gates updated.xlsx
@@ -7270,10 +7270,10 @@
       </c>
     </row>
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A137" s="1" t="s">
+      <c r="A137" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B137" s="2" t="n">
+      <c r="B137" s="8" t="n">
         <v>46</v>
       </c>
       <c r="C137" s="23" t="str">
@@ -7534,10 +7534,10 @@
       </c>
     </row>
     <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A152" s="1" t="s">
+      <c r="A152" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B152" s="2" t="n">
+      <c r="B152" s="8" t="n">
         <v>62</v>
       </c>
       <c r="C152" s="24" t="str">
@@ -7552,10 +7552,10 @@
       </c>
     </row>
     <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A153" s="1" t="s">
+      <c r="A153" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B153" s="2" t="n">
+      <c r="B153" s="8" t="n">
         <v>63</v>
       </c>
       <c r="C153" s="24" t="str">
@@ -7570,10 +7570,10 @@
       </c>
     </row>
     <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A154" s="1" t="s">
+      <c r="A154" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B154" s="2" t="n">
+      <c r="B154" s="8" t="n">
         <v>64</v>
       </c>
       <c r="C154" s="24" t="str">
@@ -7588,10 +7588,10 @@
       </c>
     </row>
     <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A155" s="1" t="s">
+      <c r="A155" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B155" s="2" t="n">
+      <c r="B155" s="8" t="n">
         <v>65</v>
       </c>
       <c r="C155" s="24" t="str">
@@ -7606,10 +7606,10 @@
       </c>
     </row>
     <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A156" s="1" t="s">
+      <c r="A156" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B156" s="2" t="n">
+      <c r="B156" s="8" t="n">
         <v>66</v>
       </c>
       <c r="C156" s="24" t="str">
@@ -7624,10 +7624,10 @@
       </c>
     </row>
     <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A157" s="1" t="s">
+      <c r="A157" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B157" s="2" t="n">
+      <c r="B157" s="8" t="n">
         <v>67</v>
       </c>
       <c r="C157" s="24" t="str">
@@ -7642,10 +7642,10 @@
       </c>
     </row>
     <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A158" s="1" t="s">
+      <c r="A158" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B158" s="2" t="n">
+      <c r="B158" s="8" t="n">
         <v>68</v>
       </c>
       <c r="C158" s="24" t="str">
@@ -7675,10 +7675,10 @@
       </c>
     </row>
     <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A160" s="1" t="s">
+      <c r="A160" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B160" s="2" t="n">
+      <c r="B160" s="8" t="n">
         <v>70</v>
       </c>
       <c r="C160" s="25" t="str">
@@ -7693,10 +7693,10 @@
       </c>
     </row>
     <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A161" s="1" t="s">
+      <c r="A161" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B161" s="2" t="n">
+      <c r="B161" s="8" t="n">
         <v>71</v>
       </c>
       <c r="C161" s="25" t="str">
@@ -7762,10 +7762,10 @@
       </c>
     </row>
     <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A165" s="1" t="s">
+      <c r="A165" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B165" s="2" t="n">
+      <c r="B165" s="8" t="n">
         <v>75</v>
       </c>
       <c r="C165" s="25" t="str">
@@ -7780,10 +7780,10 @@
       </c>
     </row>
     <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A166" s="1" t="s">
+      <c r="A166" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B166" s="2" t="n">
+      <c r="B166" s="8" t="n">
         <v>76</v>
       </c>
       <c r="C166" s="23" t="str">
@@ -7795,10 +7795,10 @@
       </c>
     </row>
     <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A167" s="1" t="s">
+      <c r="A167" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B167" s="2" t="n">
+      <c r="B167" s="8" t="n">
         <v>77</v>
       </c>
       <c r="C167" s="23" t="str">
@@ -7810,10 +7810,10 @@
       </c>
     </row>
     <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A168" s="1" t="s">
+      <c r="A168" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B168" s="2" t="n">
+      <c r="B168" s="8" t="n">
         <v>78</v>
       </c>
       <c r="C168" s="25" t="str">
@@ -7828,10 +7828,10 @@
       </c>
     </row>
     <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A169" s="1" t="s">
+      <c r="A169" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B169" s="2" t="n">
+      <c r="B169" s="8" t="n">
         <v>79</v>
       </c>
       <c r="C169" s="25" t="str">
@@ -7864,10 +7864,10 @@
       </c>
     </row>
     <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A171" s="1" t="s">
+      <c r="A171" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B171" s="2" t="n">
+      <c r="B171" s="8" t="n">
         <v>81</v>
       </c>
       <c r="C171" s="25" t="str">
@@ -7882,10 +7882,10 @@
       </c>
     </row>
     <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A172" s="1" t="s">
+      <c r="A172" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B172" s="2" t="n">
+      <c r="B172" s="8" t="n">
         <v>82</v>
       </c>
       <c r="C172" s="25" t="str">
@@ -7900,10 +7900,10 @@
       </c>
     </row>
     <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A173" s="1" t="s">
+      <c r="A173" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B173" s="2" t="n">
+      <c r="B173" s="8" t="n">
         <v>83</v>
       </c>
       <c r="C173" s="25" t="str">
@@ -7954,10 +7954,10 @@
       </c>
     </row>
     <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A176" s="1" t="s">
+      <c r="A176" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B176" s="2" t="n">
+      <c r="B176" s="8" t="n">
         <v>86</v>
       </c>
       <c r="C176" s="23" t="str">
@@ -7969,10 +7969,10 @@
       </c>
     </row>
     <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A177" s="1" t="s">
+      <c r="A177" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B177" s="2" t="n">
+      <c r="B177" s="8" t="n">
         <v>87</v>
       </c>
       <c r="C177" s="24" t="str">
@@ -7987,10 +7987,10 @@
       </c>
     </row>
     <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A178" s="1" t="s">
+      <c r="A178" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B178" s="2" t="n">
+      <c r="B178" s="8" t="n">
         <v>88</v>
       </c>
       <c r="C178" s="25" t="str">
@@ -8005,10 +8005,10 @@
       </c>
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A179" s="1" t="s">
+      <c r="A179" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B179" s="2" t="n">
+      <c r="B179" s="8" t="n">
         <v>89</v>
       </c>
       <c r="C179" s="10" t="s">
@@ -8087,10 +8087,10 @@
       </c>
     </row>
     <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A184" s="1" t="s">
+      <c r="A184" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B184" s="2" t="n">
+      <c r="B184" s="8" t="n">
         <v>94</v>
       </c>
       <c r="C184" s="10" t="s">
@@ -8635,10 +8635,10 @@
       </c>
     </row>
     <row r="213" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A213" s="1" t="s">
+      <c r="A213" s="7" t="s">
         <v>190</v>
       </c>
-      <c r="B213" s="2" t="n">
+      <c r="B213" s="8" t="n">
         <v>13</v>
       </c>
       <c r="C213" s="23" t="str">
@@ -12868,10 +12868,10 @@
       </c>
     </row>
     <row r="446" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A446" s="1" t="s">
+      <c r="A446" s="7" t="s">
         <v>325</v>
       </c>
-      <c r="B446" s="2" t="n">
+      <c r="B446" s="8" t="n">
         <v>29</v>
       </c>
       <c r="C446" s="37" t="str">
@@ -13344,10 +13344,10 @@
       </c>
     </row>
     <row r="471" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A471" s="1" t="s">
+      <c r="A471" s="7" t="s">
         <v>337</v>
       </c>
-      <c r="B471" s="2" t="n">
+      <c r="B471" s="8" t="n">
         <v>17</v>
       </c>
       <c r="C471" s="25" t="str">
@@ -13521,10 +13521,10 @@
       </c>
     </row>
     <row r="481" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A481" s="1" t="s">
+      <c r="A481" s="7" t="s">
         <v>337</v>
       </c>
-      <c r="B481" s="2" t="n">
+      <c r="B481" s="8" t="n">
         <v>27</v>
       </c>
       <c r="C481" s="25" t="str">
@@ -14350,10 +14350,10 @@
       </c>
     </row>
     <row r="530" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A530" s="1" t="s">
+      <c r="A530" s="7" t="s">
         <v>337</v>
       </c>
-      <c r="B530" s="2" t="n">
+      <c r="B530" s="8" t="n">
         <v>88</v>
       </c>
       <c r="C530" s="37" t="str">

</xml_diff>

<commit_message>
- Finished up the CHR Ax bits.
</commit_message>
<xml_diff>
--- a/list of gates updated.xlsx
+++ b/list of gates updated.xlsx
@@ -31295,11 +31295,11 @@
         <v>1164</v>
       </c>
       <c r="B1517" s="8" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="C1517" s="71" t="str">
         <f aca="false">CONCATENATE(A1517,B1517)</f>
-        <v>AX0</v>
+        <v>AX18</v>
       </c>
       <c r="D1517" s="1" t="n">
         <v>15</v>
@@ -31312,10 +31312,10 @@
       </c>
     </row>
     <row r="1518" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1518" s="1" t="s">
+      <c r="A1518" s="7" t="s">
         <v>1166</v>
       </c>
-      <c r="B1518" s="2" t="n">
+      <c r="B1518" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C1518" s="71" t="str">
@@ -31330,10 +31330,10 @@
       </c>
     </row>
     <row r="1519" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1519" s="1" t="s">
+      <c r="A1519" s="7" t="s">
         <v>1166</v>
       </c>
-      <c r="B1519" s="2" t="n">
+      <c r="B1519" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C1519" s="71" t="str">
@@ -31348,10 +31348,10 @@
       </c>
     </row>
     <row r="1520" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1520" s="1" t="s">
+      <c r="A1520" s="7" t="s">
         <v>1166</v>
       </c>
-      <c r="B1520" s="2" t="n">
+      <c r="B1520" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C1520" s="71" t="str">
@@ -31366,10 +31366,10 @@
       </c>
     </row>
     <row r="1521" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1521" s="1" t="s">
+      <c r="A1521" s="7" t="s">
         <v>1166</v>
       </c>
-      <c r="B1521" s="2" t="n">
+      <c r="B1521" s="8" t="n">
         <v>4</v>
       </c>
       <c r="C1521" s="71" t="str">
@@ -31384,10 +31384,10 @@
       </c>
     </row>
     <row r="1522" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1522" s="1" t="s">
+      <c r="A1522" s="7" t="s">
         <v>1166</v>
       </c>
-      <c r="B1522" s="2" t="n">
+      <c r="B1522" s="8" t="n">
         <v>5</v>
       </c>
       <c r="C1522" s="71" t="str">
@@ -31402,10 +31402,10 @@
       </c>
     </row>
     <row r="1523" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1523" s="1" t="s">
+      <c r="A1523" s="7" t="s">
         <v>1166</v>
       </c>
-      <c r="B1523" s="2" t="n">
+      <c r="B1523" s="8" t="n">
         <v>6</v>
       </c>
       <c r="C1523" s="71" t="str">
@@ -31420,10 +31420,10 @@
       </c>
     </row>
     <row r="1524" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1524" s="1" t="s">
+      <c r="A1524" s="7" t="s">
         <v>1166</v>
       </c>
-      <c r="B1524" s="2" t="n">
+      <c r="B1524" s="8" t="n">
         <v>7</v>
       </c>
       <c r="C1524" s="71" t="str">
@@ -31438,10 +31438,10 @@
       </c>
     </row>
     <row r="1525" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1525" s="1" t="s">
+      <c r="A1525" s="7" t="s">
         <v>1166</v>
       </c>
-      <c r="B1525" s="2" t="n">
+      <c r="B1525" s="8" t="n">
         <v>8</v>
       </c>
       <c r="C1525" s="71" t="str">
@@ -31456,10 +31456,10 @@
       </c>
     </row>
     <row r="1526" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1526" s="1" t="s">
+      <c r="A1526" s="7" t="s">
         <v>1166</v>
       </c>
-      <c r="B1526" s="2" t="n">
+      <c r="B1526" s="8" t="n">
         <v>9</v>
       </c>
       <c r="C1526" s="71" t="str">
@@ -31474,10 +31474,10 @@
       </c>
     </row>
     <row r="1527" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1527" s="1" t="s">
+      <c r="A1527" s="7" t="s">
         <v>1166</v>
       </c>
-      <c r="B1527" s="2" t="n">
+      <c r="B1527" s="8" t="n">
         <v>10</v>
       </c>
       <c r="C1527" s="71" t="str">
@@ -31492,10 +31492,10 @@
       </c>
     </row>
     <row r="1528" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1528" s="1" t="s">
+      <c r="A1528" s="7" t="s">
         <v>1166</v>
       </c>
-      <c r="B1528" s="2" t="n">
+      <c r="B1528" s="8" t="n">
         <v>11</v>
       </c>
       <c r="C1528" s="71" t="str">
@@ -31510,10 +31510,10 @@
       </c>
     </row>
     <row r="1529" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1529" s="1" t="s">
+      <c r="A1529" s="7" t="s">
         <v>1166</v>
       </c>
-      <c r="B1529" s="2" t="n">
+      <c r="B1529" s="8" t="n">
         <v>12</v>
       </c>
       <c r="C1529" s="71" t="str">
@@ -31528,10 +31528,10 @@
       </c>
     </row>
     <row r="1530" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1530" s="1" t="s">
+      <c r="A1530" s="7" t="s">
         <v>1166</v>
       </c>
-      <c r="B1530" s="2" t="n">
+      <c r="B1530" s="8" t="n">
         <v>13</v>
       </c>
       <c r="C1530" s="71" t="str">
@@ -31546,10 +31546,10 @@
       </c>
     </row>
     <row r="1531" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1531" s="1" t="s">
+      <c r="A1531" s="7" t="s">
         <v>1166</v>
       </c>
-      <c r="B1531" s="2" t="n">
+      <c r="B1531" s="8" t="n">
         <v>14</v>
       </c>
       <c r="C1531" s="71" t="str">
@@ -31564,10 +31564,10 @@
       </c>
     </row>
     <row r="1532" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1532" s="1" t="s">
+      <c r="A1532" s="7" t="s">
         <v>1166</v>
       </c>
-      <c r="B1532" s="2" t="n">
+      <c r="B1532" s="8" t="n">
         <v>15</v>
       </c>
       <c r="C1532" s="71" t="str">
@@ -31582,10 +31582,10 @@
       </c>
     </row>
     <row r="1533" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1533" s="1" t="s">
+      <c r="A1533" s="7" t="s">
         <v>1166</v>
       </c>
-      <c r="B1533" s="2" t="n">
+      <c r="B1533" s="8" t="n">
         <v>16</v>
       </c>
       <c r="C1533" s="71" t="str">
@@ -31600,10 +31600,10 @@
       </c>
     </row>
     <row r="1534" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1534" s="1" t="s">
+      <c r="A1534" s="7" t="s">
         <v>1166</v>
       </c>
-      <c r="B1534" s="2" t="n">
+      <c r="B1534" s="8" t="n">
         <v>17</v>
       </c>
       <c r="C1534" s="71" t="str">
@@ -31621,10 +31621,10 @@
       </c>
     </row>
     <row r="1535" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1535" s="1" t="s">
+      <c r="A1535" s="7" t="s">
         <v>1168</v>
       </c>
-      <c r="B1535" s="2" t="n">
+      <c r="B1535" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C1535" s="71" t="str">
@@ -31639,10 +31639,10 @@
       </c>
     </row>
     <row r="1536" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1536" s="1" t="s">
+      <c r="A1536" s="7" t="s">
         <v>1168</v>
       </c>
-      <c r="B1536" s="2" t="n">
+      <c r="B1536" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C1536" s="71" t="str">
@@ -31657,10 +31657,10 @@
       </c>
     </row>
     <row r="1537" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1537" s="1" t="s">
+      <c r="A1537" s="7" t="s">
         <v>1168</v>
       </c>
-      <c r="B1537" s="2" t="n">
+      <c r="B1537" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C1537" s="71" t="str">
@@ -31675,10 +31675,10 @@
       </c>
     </row>
     <row r="1538" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1538" s="1" t="s">
+      <c r="A1538" s="7" t="s">
         <v>1168</v>
       </c>
-      <c r="B1538" s="2" t="n">
+      <c r="B1538" s="8" t="n">
         <v>4</v>
       </c>
       <c r="C1538" s="71" t="str">
@@ -31693,10 +31693,10 @@
       </c>
     </row>
     <row r="1539" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1539" s="1" t="s">
+      <c r="A1539" s="7" t="s">
         <v>1168</v>
       </c>
-      <c r="B1539" s="2" t="n">
+      <c r="B1539" s="8" t="n">
         <v>5</v>
       </c>
       <c r="C1539" s="71" t="str">
@@ -31711,10 +31711,10 @@
       </c>
     </row>
     <row r="1540" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1540" s="1" t="s">
+      <c r="A1540" s="7" t="s">
         <v>1168</v>
       </c>
-      <c r="B1540" s="2" t="n">
+      <c r="B1540" s="8" t="n">
         <v>6</v>
       </c>
       <c r="C1540" s="71" t="str">
@@ -31729,10 +31729,10 @@
       </c>
     </row>
     <row r="1541" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1541" s="1" t="s">
+      <c r="A1541" s="7" t="s">
         <v>1168</v>
       </c>
-      <c r="B1541" s="2" t="n">
+      <c r="B1541" s="8" t="n">
         <v>7</v>
       </c>
       <c r="C1541" s="71" t="str">
@@ -31747,10 +31747,10 @@
       </c>
     </row>
     <row r="1542" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1542" s="1" t="s">
+      <c r="A1542" s="7" t="s">
         <v>1168</v>
       </c>
-      <c r="B1542" s="2" t="n">
+      <c r="B1542" s="8" t="n">
         <v>8</v>
       </c>
       <c r="C1542" s="71" t="str">
@@ -31765,10 +31765,10 @@
       </c>
     </row>
     <row r="1543" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1543" s="1" t="s">
+      <c r="A1543" s="7" t="s">
         <v>1168</v>
       </c>
-      <c r="B1543" s="2" t="n">
+      <c r="B1543" s="8" t="n">
         <v>9</v>
       </c>
       <c r="C1543" s="71" t="str">
@@ -31783,10 +31783,10 @@
       </c>
     </row>
     <row r="1544" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1544" s="1" t="s">
+      <c r="A1544" s="7" t="s">
         <v>1168</v>
       </c>
-      <c r="B1544" s="2" t="n">
+      <c r="B1544" s="8" t="n">
         <v>10</v>
       </c>
       <c r="C1544" s="71" t="str">
@@ -31801,10 +31801,10 @@
       </c>
     </row>
     <row r="1545" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1545" s="1" t="s">
+      <c r="A1545" s="7" t="s">
         <v>1168</v>
       </c>
-      <c r="B1545" s="2" t="n">
+      <c r="B1545" s="8" t="n">
         <v>11</v>
       </c>
       <c r="C1545" s="71" t="str">
@@ -31819,10 +31819,10 @@
       </c>
     </row>
     <row r="1546" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1546" s="1" t="s">
+      <c r="A1546" s="7" t="s">
         <v>1168</v>
       </c>
-      <c r="B1546" s="2" t="n">
+      <c r="B1546" s="8" t="n">
         <v>13</v>
       </c>
       <c r="C1546" s="71" t="str">
@@ -31837,10 +31837,10 @@
       </c>
     </row>
     <row r="1547" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1547" s="1" t="s">
+      <c r="A1547" s="7" t="s">
         <v>1168</v>
       </c>
-      <c r="B1547" s="2" t="n">
+      <c r="B1547" s="8" t="n">
         <v>14</v>
       </c>
       <c r="C1547" s="71" t="str">
@@ -31855,10 +31855,10 @@
       </c>
     </row>
     <row r="1548" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1548" s="1" t="s">
+      <c r="A1548" s="7" t="s">
         <v>1168</v>
       </c>
-      <c r="B1548" s="2" t="n">
+      <c r="B1548" s="8" t="n">
         <v>15</v>
       </c>
       <c r="C1548" s="71" t="str">
@@ -31873,10 +31873,10 @@
       </c>
     </row>
     <row r="1549" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1549" s="1" t="s">
+      <c r="A1549" s="7" t="s">
         <v>1168</v>
       </c>
-      <c r="B1549" s="2" t="n">
+      <c r="B1549" s="8" t="n">
         <v>16</v>
       </c>
       <c r="C1549" s="71" t="str">
@@ -31891,10 +31891,10 @@
       </c>
     </row>
     <row r="1550" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1550" s="1" t="s">
+      <c r="A1550" s="7" t="s">
         <v>1168</v>
       </c>
-      <c r="B1550" s="2" t="n">
+      <c r="B1550" s="8" t="n">
         <v>17</v>
       </c>
       <c r="C1550" s="71" t="str">
@@ -31912,10 +31912,10 @@
       </c>
     </row>
     <row r="1551" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1551" s="1" t="s">
+      <c r="A1551" s="7" t="s">
         <v>1170</v>
       </c>
-      <c r="B1551" s="2" t="n">
+      <c r="B1551" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C1551" s="74" t="str">
@@ -31930,10 +31930,10 @@
       </c>
     </row>
     <row r="1552" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1552" s="1" t="s">
+      <c r="A1552" s="7" t="s">
         <v>1170</v>
       </c>
-      <c r="B1552" s="2" t="n">
+      <c r="B1552" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C1552" s="74" t="str">
@@ -31948,10 +31948,10 @@
       </c>
     </row>
     <row r="1553" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1553" s="1" t="s">
+      <c r="A1553" s="7" t="s">
         <v>1170</v>
       </c>
-      <c r="B1553" s="2" t="n">
+      <c r="B1553" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C1553" s="74" t="str">
@@ -31966,10 +31966,10 @@
       </c>
     </row>
     <row r="1554" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1554" s="1" t="s">
+      <c r="A1554" s="7" t="s">
         <v>1170</v>
       </c>
-      <c r="B1554" s="2" t="n">
+      <c r="B1554" s="8" t="n">
         <v>4</v>
       </c>
       <c r="C1554" s="74" t="str">
@@ -31984,10 +31984,10 @@
       </c>
     </row>
     <row r="1555" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1555" s="1" t="s">
+      <c r="A1555" s="7" t="s">
         <v>1170</v>
       </c>
-      <c r="B1555" s="2" t="n">
+      <c r="B1555" s="8" t="n">
         <v>5</v>
       </c>
       <c r="C1555" s="74" t="str">
@@ -32002,10 +32002,10 @@
       </c>
     </row>
     <row r="1556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1556" s="1" t="s">
+      <c r="A1556" s="7" t="s">
         <v>1170</v>
       </c>
-      <c r="B1556" s="2" t="n">
+      <c r="B1556" s="8" t="n">
         <v>6</v>
       </c>
       <c r="C1556" s="74" t="str">
@@ -32020,10 +32020,10 @@
       </c>
     </row>
     <row r="1557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1557" s="1" t="s">
+      <c r="A1557" s="7" t="s">
         <v>1170</v>
       </c>
-      <c r="B1557" s="2" t="n">
+      <c r="B1557" s="8" t="n">
         <v>7</v>
       </c>
       <c r="C1557" s="74" t="str">
@@ -32038,10 +32038,10 @@
       </c>
     </row>
     <row r="1558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1558" s="1" t="s">
+      <c r="A1558" s="7" t="s">
         <v>1170</v>
       </c>
-      <c r="B1558" s="2" t="n">
+      <c r="B1558" s="8" t="n">
         <v>8</v>
       </c>
       <c r="C1558" s="74" t="str">
@@ -32056,10 +32056,10 @@
       </c>
     </row>
     <row r="1559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1559" s="1" t="s">
+      <c r="A1559" s="7" t="s">
         <v>1170</v>
       </c>
-      <c r="B1559" s="2" t="n">
+      <c r="B1559" s="8" t="n">
         <v>9</v>
       </c>
       <c r="C1559" s="74" t="str">
@@ -32074,10 +32074,10 @@
       </c>
     </row>
     <row r="1560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1560" s="1" t="s">
+      <c r="A1560" s="7" t="s">
         <v>1170</v>
       </c>
-      <c r="B1560" s="2" t="n">
+      <c r="B1560" s="8" t="n">
         <v>10</v>
       </c>
       <c r="C1560" s="74" t="str">
@@ -32092,10 +32092,10 @@
       </c>
     </row>
     <row r="1561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1561" s="1" t="s">
+      <c r="A1561" s="7" t="s">
         <v>1170</v>
       </c>
-      <c r="B1561" s="2" t="n">
+      <c r="B1561" s="8" t="n">
         <v>11</v>
       </c>
       <c r="C1561" s="74" t="str">
@@ -32110,10 +32110,10 @@
       </c>
     </row>
     <row r="1562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1562" s="1" t="s">
+      <c r="A1562" s="7" t="s">
         <v>1170</v>
       </c>
-      <c r="B1562" s="2" t="n">
+      <c r="B1562" s="8" t="n">
         <v>12</v>
       </c>
       <c r="C1562" s="74" t="str">
@@ -32128,10 +32128,10 @@
       </c>
     </row>
     <row r="1563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1563" s="1" t="s">
+      <c r="A1563" s="7" t="s">
         <v>1170</v>
       </c>
-      <c r="B1563" s="2" t="n">
+      <c r="B1563" s="8" t="n">
         <v>13</v>
       </c>
       <c r="C1563" s="74" t="str">
@@ -32146,10 +32146,10 @@
       </c>
     </row>
     <row r="1564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1564" s="1" t="s">
+      <c r="A1564" s="7" t="s">
         <v>1170</v>
       </c>
-      <c r="B1564" s="2" t="n">
+      <c r="B1564" s="8" t="n">
         <v>14</v>
       </c>
       <c r="C1564" s="74" t="str">
@@ -32164,10 +32164,10 @@
       </c>
     </row>
     <row r="1565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1565" s="1" t="s">
+      <c r="A1565" s="7" t="s">
         <v>1170</v>
       </c>
-      <c r="B1565" s="2" t="n">
+      <c r="B1565" s="8" t="n">
         <v>15</v>
       </c>
       <c r="C1565" s="74" t="str">
@@ -32182,10 +32182,10 @@
       </c>
     </row>
     <row r="1566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1566" s="1" t="s">
+      <c r="A1566" s="7" t="s">
         <v>1170</v>
       </c>
-      <c r="B1566" s="2" t="n">
+      <c r="B1566" s="8" t="n">
         <v>16</v>
       </c>
       <c r="C1566" s="74" t="str">
@@ -32200,10 +32200,10 @@
       </c>
     </row>
     <row r="1567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1567" s="1" t="s">
+      <c r="A1567" s="7" t="s">
         <v>1170</v>
       </c>
-      <c r="B1567" s="2" t="n">
+      <c r="B1567" s="8" t="n">
         <v>17</v>
       </c>
       <c r="C1567" s="74" t="str">
@@ -32221,10 +32221,10 @@
       </c>
     </row>
     <row r="1568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1568" s="1" t="s">
+      <c r="A1568" s="7" t="s">
         <v>1172</v>
       </c>
-      <c r="B1568" s="2" t="n">
+      <c r="B1568" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C1568" s="74" t="str">
@@ -32239,10 +32239,10 @@
       </c>
     </row>
     <row r="1569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1569" s="1" t="s">
+      <c r="A1569" s="7" t="s">
         <v>1172</v>
       </c>
-      <c r="B1569" s="2" t="n">
+      <c r="B1569" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C1569" s="74" t="str">
@@ -32257,10 +32257,10 @@
       </c>
     </row>
     <row r="1570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1570" s="1" t="s">
+      <c r="A1570" s="7" t="s">
         <v>1172</v>
       </c>
-      <c r="B1570" s="2" t="n">
+      <c r="B1570" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C1570" s="74" t="str">
@@ -32275,10 +32275,10 @@
       </c>
     </row>
     <row r="1571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1571" s="1" t="s">
+      <c r="A1571" s="7" t="s">
         <v>1172</v>
       </c>
-      <c r="B1571" s="2" t="n">
+      <c r="B1571" s="8" t="n">
         <v>4</v>
       </c>
       <c r="C1571" s="74" t="str">
@@ -32293,10 +32293,10 @@
       </c>
     </row>
     <row r="1572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1572" s="1" t="s">
+      <c r="A1572" s="7" t="s">
         <v>1172</v>
       </c>
-      <c r="B1572" s="2" t="n">
+      <c r="B1572" s="8" t="n">
         <v>5</v>
       </c>
       <c r="C1572" s="74" t="str">
@@ -32311,10 +32311,10 @@
       </c>
     </row>
     <row r="1573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1573" s="1" t="s">
+      <c r="A1573" s="7" t="s">
         <v>1172</v>
       </c>
-      <c r="B1573" s="2" t="n">
+      <c r="B1573" s="8" t="n">
         <v>6</v>
       </c>
       <c r="C1573" s="74" t="str">
@@ -32329,10 +32329,10 @@
       </c>
     </row>
     <row r="1574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1574" s="1" t="s">
+      <c r="A1574" s="7" t="s">
         <v>1172</v>
       </c>
-      <c r="B1574" s="2" t="n">
+      <c r="B1574" s="8" t="n">
         <v>7</v>
       </c>
       <c r="C1574" s="74" t="str">
@@ -32347,10 +32347,10 @@
       </c>
     </row>
     <row r="1575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1575" s="1" t="s">
+      <c r="A1575" s="7" t="s">
         <v>1172</v>
       </c>
-      <c r="B1575" s="2" t="n">
+      <c r="B1575" s="8" t="n">
         <v>8</v>
       </c>
       <c r="C1575" s="74" t="str">
@@ -32365,10 +32365,10 @@
       </c>
     </row>
     <row r="1576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1576" s="1" t="s">
+      <c r="A1576" s="7" t="s">
         <v>1172</v>
       </c>
-      <c r="B1576" s="2" t="n">
+      <c r="B1576" s="8" t="n">
         <v>9</v>
       </c>
       <c r="C1576" s="74" t="str">
@@ -32383,10 +32383,10 @@
       </c>
     </row>
     <row r="1577" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1577" s="1" t="s">
+      <c r="A1577" s="7" t="s">
         <v>1172</v>
       </c>
-      <c r="B1577" s="2" t="n">
+      <c r="B1577" s="8" t="n">
         <v>10</v>
       </c>
       <c r="C1577" s="74" t="str">
@@ -32401,10 +32401,10 @@
       </c>
     </row>
     <row r="1578" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1578" s="1" t="s">
+      <c r="A1578" s="7" t="s">
         <v>1172</v>
       </c>
-      <c r="B1578" s="2" t="n">
+      <c r="B1578" s="8" t="n">
         <v>11</v>
       </c>
       <c r="C1578" s="74" t="str">
@@ -32419,10 +32419,10 @@
       </c>
     </row>
     <row r="1579" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1579" s="1" t="s">
+      <c r="A1579" s="7" t="s">
         <v>1172</v>
       </c>
-      <c r="B1579" s="2" t="n">
+      <c r="B1579" s="8" t="n">
         <v>12</v>
       </c>
       <c r="C1579" s="74" t="str">
@@ -32437,10 +32437,10 @@
       </c>
     </row>
     <row r="1580" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1580" s="1" t="s">
+      <c r="A1580" s="7" t="s">
         <v>1172</v>
       </c>
-      <c r="B1580" s="2" t="n">
+      <c r="B1580" s="8" t="n">
         <v>13</v>
       </c>
       <c r="C1580" s="74" t="str">
@@ -32455,10 +32455,10 @@
       </c>
     </row>
     <row r="1581" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1581" s="1" t="s">
+      <c r="A1581" s="7" t="s">
         <v>1172</v>
       </c>
-      <c r="B1581" s="2" t="n">
+      <c r="B1581" s="8" t="n">
         <v>14</v>
       </c>
       <c r="C1581" s="74" t="str">
@@ -32473,10 +32473,10 @@
       </c>
     </row>
     <row r="1582" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1582" s="1" t="s">
+      <c r="A1582" s="7" t="s">
         <v>1172</v>
       </c>
-      <c r="B1582" s="2" t="n">
+      <c r="B1582" s="8" t="n">
         <v>15</v>
       </c>
       <c r="C1582" s="74" t="str">
@@ -32491,10 +32491,10 @@
       </c>
     </row>
     <row r="1583" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1583" s="1" t="s">
+      <c r="A1583" s="7" t="s">
         <v>1172</v>
       </c>
-      <c r="B1583" s="2" t="n">
+      <c r="B1583" s="8" t="n">
         <v>16</v>
       </c>
       <c r="C1583" s="74" t="str">
@@ -32509,10 +32509,10 @@
       </c>
     </row>
     <row r="1584" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1584" s="1" t="s">
+      <c r="A1584" s="7" t="s">
         <v>1172</v>
       </c>
-      <c r="B1584" s="2" t="n">
+      <c r="B1584" s="8" t="n">
         <v>17</v>
       </c>
       <c r="C1584" s="74" t="str">
@@ -32530,10 +32530,10 @@
       </c>
     </row>
     <row r="1585" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1585" s="1" t="s">
+      <c r="A1585" s="7" t="s">
         <v>1174</v>
       </c>
-      <c r="B1585" s="2" t="n">
+      <c r="B1585" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C1585" s="74" t="str">
@@ -32548,10 +32548,10 @@
       </c>
     </row>
     <row r="1586" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1586" s="1" t="s">
+      <c r="A1586" s="7" t="s">
         <v>1174</v>
       </c>
-      <c r="B1586" s="2" t="n">
+      <c r="B1586" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C1586" s="74" t="str">
@@ -32566,10 +32566,10 @@
       </c>
     </row>
     <row r="1587" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1587" s="1" t="s">
+      <c r="A1587" s="7" t="s">
         <v>1174</v>
       </c>
-      <c r="B1587" s="2" t="n">
+      <c r="B1587" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C1587" s="74" t="str">
@@ -32584,10 +32584,10 @@
       </c>
     </row>
     <row r="1588" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1588" s="1" t="s">
+      <c r="A1588" s="7" t="s">
         <v>1174</v>
       </c>
-      <c r="B1588" s="2" t="n">
+      <c r="B1588" s="8" t="n">
         <v>4</v>
       </c>
       <c r="C1588" s="74" t="str">
@@ -32602,10 +32602,10 @@
       </c>
     </row>
     <row r="1589" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1589" s="1" t="s">
+      <c r="A1589" s="7" t="s">
         <v>1174</v>
       </c>
-      <c r="B1589" s="2" t="n">
+      <c r="B1589" s="8" t="n">
         <v>5</v>
       </c>
       <c r="C1589" s="74" t="str">
@@ -32620,10 +32620,10 @@
       </c>
     </row>
     <row r="1590" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1590" s="1" t="s">
+      <c r="A1590" s="7" t="s">
         <v>1174</v>
       </c>
-      <c r="B1590" s="2" t="n">
+      <c r="B1590" s="8" t="n">
         <v>6</v>
       </c>
       <c r="C1590" s="74" t="str">
@@ -32638,10 +32638,10 @@
       </c>
     </row>
     <row r="1591" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1591" s="1" t="s">
+      <c r="A1591" s="7" t="s">
         <v>1174</v>
       </c>
-      <c r="B1591" s="2" t="n">
+      <c r="B1591" s="8" t="n">
         <v>7</v>
       </c>
       <c r="C1591" s="74" t="str">
@@ -32656,10 +32656,10 @@
       </c>
     </row>
     <row r="1592" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1592" s="1" t="s">
+      <c r="A1592" s="7" t="s">
         <v>1174</v>
       </c>
-      <c r="B1592" s="2" t="n">
+      <c r="B1592" s="8" t="n">
         <v>8</v>
       </c>
       <c r="C1592" s="74" t="str">
@@ -32674,10 +32674,10 @@
       </c>
     </row>
     <row r="1593" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1593" s="1" t="s">
+      <c r="A1593" s="7" t="s">
         <v>1174</v>
       </c>
-      <c r="B1593" s="2" t="n">
+      <c r="B1593" s="8" t="n">
         <v>9</v>
       </c>
       <c r="C1593" s="74" t="str">
@@ -32692,10 +32692,10 @@
       </c>
     </row>
     <row r="1594" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1594" s="1" t="s">
+      <c r="A1594" s="7" t="s">
         <v>1174</v>
       </c>
-      <c r="B1594" s="2" t="n">
+      <c r="B1594" s="8" t="n">
         <v>10</v>
       </c>
       <c r="C1594" s="74" t="str">
@@ -32710,10 +32710,10 @@
       </c>
     </row>
     <row r="1595" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1595" s="1" t="s">
+      <c r="A1595" s="7" t="s">
         <v>1174</v>
       </c>
-      <c r="B1595" s="2" t="n">
+      <c r="B1595" s="8" t="n">
         <v>11</v>
       </c>
       <c r="C1595" s="74" t="str">
@@ -32728,10 +32728,10 @@
       </c>
     </row>
     <row r="1596" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1596" s="1" t="s">
+      <c r="A1596" s="7" t="s">
         <v>1174</v>
       </c>
-      <c r="B1596" s="2" t="n">
+      <c r="B1596" s="8" t="n">
         <v>12</v>
       </c>
       <c r="C1596" s="74" t="str">
@@ -32746,10 +32746,10 @@
       </c>
     </row>
     <row r="1597" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1597" s="1" t="s">
+      <c r="A1597" s="7" t="s">
         <v>1174</v>
       </c>
-      <c r="B1597" s="2" t="n">
+      <c r="B1597" s="8" t="n">
         <v>13</v>
       </c>
       <c r="C1597" s="74" t="str">
@@ -32764,10 +32764,10 @@
       </c>
     </row>
     <row r="1598" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1598" s="1" t="s">
+      <c r="A1598" s="7" t="s">
         <v>1174</v>
       </c>
-      <c r="B1598" s="2" t="n">
+      <c r="B1598" s="8" t="n">
         <v>14</v>
       </c>
       <c r="C1598" s="74" t="str">
@@ -32782,10 +32782,10 @@
       </c>
     </row>
     <row r="1599" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1599" s="1" t="s">
+      <c r="A1599" s="7" t="s">
         <v>1174</v>
       </c>
-      <c r="B1599" s="2" t="n">
+      <c r="B1599" s="8" t="n">
         <v>15</v>
       </c>
       <c r="C1599" s="74" t="str">
@@ -32800,10 +32800,10 @@
       </c>
     </row>
     <row r="1600" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1600" s="1" t="s">
+      <c r="A1600" s="7" t="s">
         <v>1174</v>
       </c>
-      <c r="B1600" s="2" t="n">
+      <c r="B1600" s="8" t="n">
         <v>16</v>
       </c>
       <c r="C1600" s="74" t="str">
@@ -32818,10 +32818,10 @@
       </c>
     </row>
     <row r="1601" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1601" s="1" t="s">
+      <c r="A1601" s="7" t="s">
         <v>1174</v>
       </c>
-      <c r="B1601" s="2" t="n">
+      <c r="B1601" s="8" t="n">
         <v>17</v>
       </c>
       <c r="C1601" s="74" t="str">
@@ -32839,10 +32839,10 @@
       </c>
     </row>
     <row r="1602" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1602" s="1" t="s">
+      <c r="A1602" s="7" t="s">
         <v>1176</v>
       </c>
-      <c r="B1602" s="2" t="n">
+      <c r="B1602" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C1602" s="74" t="str">
@@ -32857,10 +32857,10 @@
       </c>
     </row>
     <row r="1603" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1603" s="1" t="s">
+      <c r="A1603" s="7" t="s">
         <v>1176</v>
       </c>
-      <c r="B1603" s="2" t="n">
+      <c r="B1603" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C1603" s="74" t="str">
@@ -32875,10 +32875,10 @@
       </c>
     </row>
     <row r="1604" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1604" s="1" t="s">
+      <c r="A1604" s="7" t="s">
         <v>1176</v>
       </c>
-      <c r="B1604" s="2" t="n">
+      <c r="B1604" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C1604" s="74" t="str">
@@ -32893,10 +32893,10 @@
       </c>
     </row>
     <row r="1605" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1605" s="1" t="s">
+      <c r="A1605" s="7" t="s">
         <v>1176</v>
       </c>
-      <c r="B1605" s="2" t="n">
+      <c r="B1605" s="8" t="n">
         <v>4</v>
       </c>
       <c r="C1605" s="74" t="str">
@@ -32911,10 +32911,10 @@
       </c>
     </row>
     <row r="1606" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1606" s="1" t="s">
+      <c r="A1606" s="7" t="s">
         <v>1176</v>
       </c>
-      <c r="B1606" s="2" t="n">
+      <c r="B1606" s="8" t="n">
         <v>5</v>
       </c>
       <c r="C1606" s="74" t="str">
@@ -32929,10 +32929,10 @@
       </c>
     </row>
     <row r="1607" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1607" s="1" t="s">
+      <c r="A1607" s="7" t="s">
         <v>1176</v>
       </c>
-      <c r="B1607" s="2" t="n">
+      <c r="B1607" s="8" t="n">
         <v>6</v>
       </c>
       <c r="C1607" s="74" t="str">
@@ -32947,10 +32947,10 @@
       </c>
     </row>
     <row r="1608" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1608" s="1" t="s">
+      <c r="A1608" s="7" t="s">
         <v>1176</v>
       </c>
-      <c r="B1608" s="2" t="n">
+      <c r="B1608" s="8" t="n">
         <v>7</v>
       </c>
       <c r="C1608" s="74" t="str">
@@ -32965,10 +32965,10 @@
       </c>
     </row>
     <row r="1609" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1609" s="1" t="s">
+      <c r="A1609" s="7" t="s">
         <v>1176</v>
       </c>
-      <c r="B1609" s="2" t="n">
+      <c r="B1609" s="8" t="n">
         <v>8</v>
       </c>
       <c r="C1609" s="74" t="str">
@@ -32983,10 +32983,10 @@
       </c>
     </row>
     <row r="1610" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1610" s="1" t="s">
+      <c r="A1610" s="7" t="s">
         <v>1176</v>
       </c>
-      <c r="B1610" s="2" t="n">
+      <c r="B1610" s="8" t="n">
         <v>9</v>
       </c>
       <c r="C1610" s="74" t="str">
@@ -33001,10 +33001,10 @@
       </c>
     </row>
     <row r="1611" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1611" s="1" t="s">
+      <c r="A1611" s="7" t="s">
         <v>1176</v>
       </c>
-      <c r="B1611" s="2" t="n">
+      <c r="B1611" s="8" t="n">
         <v>10</v>
       </c>
       <c r="C1611" s="74" t="str">
@@ -33019,10 +33019,10 @@
       </c>
     </row>
     <row r="1612" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1612" s="1" t="s">
+      <c r="A1612" s="7" t="s">
         <v>1176</v>
       </c>
-      <c r="B1612" s="2" t="n">
+      <c r="B1612" s="8" t="n">
         <v>11</v>
       </c>
       <c r="C1612" s="74" t="str">
@@ -33037,10 +33037,10 @@
       </c>
     </row>
     <row r="1613" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1613" s="1" t="s">
+      <c r="A1613" s="7" t="s">
         <v>1176</v>
       </c>
-      <c r="B1613" s="2" t="n">
+      <c r="B1613" s="8" t="n">
         <v>12</v>
       </c>
       <c r="C1613" s="74" t="str">
@@ -33055,10 +33055,10 @@
       </c>
     </row>
     <row r="1614" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1614" s="1" t="s">
+      <c r="A1614" s="7" t="s">
         <v>1176</v>
       </c>
-      <c r="B1614" s="2" t="n">
+      <c r="B1614" s="8" t="n">
         <v>13</v>
       </c>
       <c r="C1614" s="74" t="str">
@@ -33073,10 +33073,10 @@
       </c>
     </row>
     <row r="1615" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1615" s="1" t="s">
+      <c r="A1615" s="7" t="s">
         <v>1176</v>
       </c>
-      <c r="B1615" s="2" t="n">
+      <c r="B1615" s="8" t="n">
         <v>14</v>
       </c>
       <c r="C1615" s="74" t="str">
@@ -33091,10 +33091,10 @@
       </c>
     </row>
     <row r="1616" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1616" s="1" t="s">
+      <c r="A1616" s="7" t="s">
         <v>1176</v>
       </c>
-      <c r="B1616" s="2" t="n">
+      <c r="B1616" s="8" t="n">
         <v>15</v>
       </c>
       <c r="C1616" s="74" t="str">
@@ -33109,10 +33109,10 @@
       </c>
     </row>
     <row r="1617" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1617" s="1" t="s">
+      <c r="A1617" s="7" t="s">
         <v>1176</v>
       </c>
-      <c r="B1617" s="2" t="n">
+      <c r="B1617" s="8" t="n">
         <v>16</v>
       </c>
       <c r="C1617" s="74" t="str">
@@ -33127,10 +33127,10 @@
       </c>
     </row>
     <row r="1618" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1618" s="1" t="s">
+      <c r="A1618" s="7" t="s">
         <v>1176</v>
       </c>
-      <c r="B1618" s="2" t="n">
+      <c r="B1618" s="8" t="n">
         <v>17</v>
       </c>
       <c r="C1618" s="74" t="str">
@@ -33148,10 +33148,10 @@
       </c>
     </row>
     <row r="1619" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1619" s="1" t="s">
+      <c r="A1619" s="7" t="s">
         <v>1178</v>
       </c>
-      <c r="B1619" s="2" t="n">
+      <c r="B1619" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C1619" s="74" t="str">
@@ -33166,10 +33166,10 @@
       </c>
     </row>
     <row r="1620" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1620" s="1" t="s">
+      <c r="A1620" s="7" t="s">
         <v>1178</v>
       </c>
-      <c r="B1620" s="2" t="n">
+      <c r="B1620" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C1620" s="74" t="str">
@@ -33184,10 +33184,10 @@
       </c>
     </row>
     <row r="1621" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1621" s="1" t="s">
+      <c r="A1621" s="7" t="s">
         <v>1178</v>
       </c>
-      <c r="B1621" s="2" t="n">
+      <c r="B1621" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C1621" s="74" t="str">
@@ -33202,10 +33202,10 @@
       </c>
     </row>
     <row r="1622" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1622" s="1" t="s">
+      <c r="A1622" s="7" t="s">
         <v>1178</v>
       </c>
-      <c r="B1622" s="2" t="n">
+      <c r="B1622" s="8" t="n">
         <v>4</v>
       </c>
       <c r="C1622" s="74" t="str">
@@ -33220,10 +33220,10 @@
       </c>
     </row>
     <row r="1623" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1623" s="1" t="s">
+      <c r="A1623" s="7" t="s">
         <v>1178</v>
       </c>
-      <c r="B1623" s="2" t="n">
+      <c r="B1623" s="8" t="n">
         <v>5</v>
       </c>
       <c r="C1623" s="74" t="str">
@@ -33238,10 +33238,10 @@
       </c>
     </row>
     <row r="1624" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1624" s="1" t="s">
+      <c r="A1624" s="7" t="s">
         <v>1178</v>
       </c>
-      <c r="B1624" s="2" t="n">
+      <c r="B1624" s="8" t="n">
         <v>6</v>
       </c>
       <c r="C1624" s="74" t="str">
@@ -33256,10 +33256,10 @@
       </c>
     </row>
     <row r="1625" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1625" s="1" t="s">
+      <c r="A1625" s="7" t="s">
         <v>1178</v>
       </c>
-      <c r="B1625" s="2" t="n">
+      <c r="B1625" s="8" t="n">
         <v>7</v>
       </c>
       <c r="C1625" s="74" t="str">
@@ -33274,10 +33274,10 @@
       </c>
     </row>
     <row r="1626" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1626" s="1" t="s">
+      <c r="A1626" s="7" t="s">
         <v>1178</v>
       </c>
-      <c r="B1626" s="2" t="n">
+      <c r="B1626" s="8" t="n">
         <v>8</v>
       </c>
       <c r="C1626" s="74" t="str">
@@ -33292,10 +33292,10 @@
       </c>
     </row>
     <row r="1627" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1627" s="1" t="s">
+      <c r="A1627" s="7" t="s">
         <v>1178</v>
       </c>
-      <c r="B1627" s="2" t="n">
+      <c r="B1627" s="8" t="n">
         <v>9</v>
       </c>
       <c r="C1627" s="74" t="str">
@@ -33310,10 +33310,10 @@
       </c>
     </row>
     <row r="1628" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1628" s="1" t="s">
+      <c r="A1628" s="7" t="s">
         <v>1178</v>
       </c>
-      <c r="B1628" s="2" t="n">
+      <c r="B1628" s="8" t="n">
         <v>10</v>
       </c>
       <c r="C1628" s="74" t="str">
@@ -33328,10 +33328,10 @@
       </c>
     </row>
     <row r="1629" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1629" s="1" t="s">
+      <c r="A1629" s="7" t="s">
         <v>1178</v>
       </c>
-      <c r="B1629" s="2" t="n">
+      <c r="B1629" s="8" t="n">
         <v>11</v>
       </c>
       <c r="C1629" s="74" t="str">
@@ -33346,10 +33346,10 @@
       </c>
     </row>
     <row r="1630" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1630" s="1" t="s">
+      <c r="A1630" s="7" t="s">
         <v>1178</v>
       </c>
-      <c r="B1630" s="2" t="n">
+      <c r="B1630" s="8" t="n">
         <v>12</v>
       </c>
       <c r="C1630" s="74" t="str">
@@ -33364,10 +33364,10 @@
       </c>
     </row>
     <row r="1631" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1631" s="1" t="s">
+      <c r="A1631" s="7" t="s">
         <v>1178</v>
       </c>
-      <c r="B1631" s="2" t="n">
+      <c r="B1631" s="8" t="n">
         <v>13</v>
       </c>
       <c r="C1631" s="74" t="str">
@@ -33382,10 +33382,10 @@
       </c>
     </row>
     <row r="1632" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1632" s="1" t="s">
+      <c r="A1632" s="7" t="s">
         <v>1178</v>
       </c>
-      <c r="B1632" s="2" t="n">
+      <c r="B1632" s="8" t="n">
         <v>14</v>
       </c>
       <c r="C1632" s="74" t="str">
@@ -33400,10 +33400,10 @@
       </c>
     </row>
     <row r="1633" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1633" s="1" t="s">
+      <c r="A1633" s="7" t="s">
         <v>1178</v>
       </c>
-      <c r="B1633" s="2" t="n">
+      <c r="B1633" s="8" t="n">
         <v>15</v>
       </c>
       <c r="C1633" s="74" t="str">
@@ -33418,10 +33418,10 @@
       </c>
     </row>
     <row r="1634" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1634" s="1" t="s">
+      <c r="A1634" s="7" t="s">
         <v>1178</v>
       </c>
-      <c r="B1634" s="2" t="n">
+      <c r="B1634" s="8" t="n">
         <v>16</v>
       </c>
       <c r="C1634" s="74" t="str">
@@ -33436,10 +33436,10 @@
       </c>
     </row>
     <row r="1635" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1635" s="1" t="s">
+      <c r="A1635" s="7" t="s">
         <v>1178</v>
       </c>
-      <c r="B1635" s="2" t="n">
+      <c r="B1635" s="8" t="n">
         <v>17</v>
       </c>
       <c r="C1635" s="74" t="str">

</xml_diff>